<commit_message>
UK v30–v32: decided edits, Humber 2100+, five framework-currency records; Open work trimmed
- UK v30: drought orders/permits noted on LEG-025 and LEG-023; JNCC Signpost series on ORG-004;
  NPS exclusion recorded on POL-050; LEG-013 Royal Assent date verified (24 Feb 2025).
- UK v31: Humber 2100+ folded into POL-045 FCERM Strategy.
- UK v32: POL-112 CBGDP, POL-113 CCRA4-IA, POL-114 CCC progress reports (series),
  POL-115 NICCAP3, POL-116 Scotland's Climate Change Plan 2026–2040; POL-004 and POL-017
  point to their successors.
- Handover Open work now lists uncompleted tasks only; the scan coverage item merged into the
  next quarterly scan; NI Nature Recovery Strategy moved to watch items.
- Climate heatmap and outstanding-issues references removed; new Data/CANONICAL_FILES_GUIDE.md.
- pending_additions.md rows resolved; status formatting normalised.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AXpUr5Jv7F4hv6YdhfHEwx
</commit_message>
<xml_diff>
--- a/Data/canonical_files/uk_climate_nature_governance.xlsx
+++ b/Data/canonical_files/uk_climate_nature_governance.xlsx
@@ -949,7 +949,7 @@
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Statutory adviser to UK Government and devolved administrations on UK-wide and international nature conservation. Forum for country NCBs (Natural England, NatureScot, NRW, NIEA) to discharge UK and international statutory responsibilities. Maintains UK Biodiversity Indicators. Advises on international conventions (CBD, CITES, Ramsar, OSPAR). No direct regulatory powers; advisory and evidence function only.</t>
+          <t>Statutory adviser to UK Government and devolved administrations on UK-wide and international nature conservation. Forum for country NCBs (Natural England, NatureScot, NRW, NIEA) to discharge UK and international statutory responsibilities. Maintains UK Biodiversity Indicators. Advises on international conventions (CBD, CITES, Ramsar, OSPAR). No direct regulatory powers; advisory and evidence function only. Publishes the Signpost report series, 'Nature, Evidence and Action' (2026), setting out evidence and policy recommendations to accelerate nature recovery, aimed primarily at the four UK governments: private investment in peatland restoration, agricultural soil restoration, monitoring and adaptation for nature recovery, and integrating nature's value into land-use decisions (cf. [POL-009] Land Use Framework). Series: https://jncc.gov.uk/our-role/the-uk/jnccs-signpost-report-series/ — held as a mention, not as records.</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
@@ -969,7 +969,7 @@
       </c>
       <c r="M5" s="5" t="inlineStr">
         <is>
-          <t>May 2026</t>
+          <t>October 2026</t>
         </is>
       </c>
       <c r="N5" s="6" t="inlineStr">
@@ -5343,7 +5343,7 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Royal Assent Jan 2025</t>
+          <t>Royal Assent 24 Feb 2025</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
@@ -6085,7 +6085,7 @@
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>Amends water company licensing; introduces resilience duties; reforms abstraction licensing; enables Ofwat to set outcome-based price controls (PR19 onwards).</t>
+          <t>Amends water company licensing; introduces resilience duties; reforms abstraction licensing; enables Ofwat to set outcome-based price controls (PR19 onwards). s.27 adds resilience to water resources management plans for England and s.28 sets the frequency of water resources management plans and drought plans (drought plans: Water Industry Act 1991 ss.39B–39C, [LEG-012]). Drought orders and drought permits themselves sit in the Water Resources Act 1991 [LEG-025].</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -6100,7 +6100,7 @@
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>May 2026</t>
+          <t>October 2026</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
@@ -6237,7 +6237,7 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>Grants EA powers over water abstraction licensing, flood risk, and water quality. Defines controlled waters and regulates discharge consents.</t>
+          <t>Grants EA powers over water abstraction licensing, flood risk, and water quality. Defines controlled waters and regulates discharge consents. Part II Chapter III (ss.73–81) is the statutory drought-response mechanism: ordinary and emergency drought orders, made by the Secretary of State on application by the Environment Agency (Natural Resources Wales in Wales) or a water undertaker, can restrict water use and modify abstractions and discharges; drought permits (s.79A) are issued by the agency itself. Individual drought orders, permits and restriction notices are not catalogued as records (decision, 11 Sep 2026).</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -6252,7 +6252,7 @@
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>May 2026</t>
+          <t>October 2026</t>
         </is>
       </c>
       <c r="N24" s="4" t="inlineStr">
@@ -9805,7 +9805,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S110"/>
+  <dimension ref="A1:S115"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="32" min="1" max="1"/>
@@ -10223,7 +10223,11 @@
           <t>[LEG-001]; [LEG-002]</t>
         </is>
       </c>
-      <c r="J5" s="5" t="n"/>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>[POL-112] Carbon Budget and Growth Delivery Plan (CBGDP)</t>
+        </is>
+      </c>
       <c r="K5" s="5" t="n"/>
       <c r="L5" s="5" t="n"/>
       <c r="M5" s="5" t="inlineStr">
@@ -10234,7 +10238,7 @@
       <c r="N5" s="5" t="inlineStr">
         <is>
           <t>Policy plan setting out government's approach to meeting CB4–CB6 carbon budgets and 2050 net-zero target. Covers 9 sectors: electricity, buildings, transport, industry, agriculture/land, aviation, shipping, waste/F-gases, fuel supply. Contains sectoral pathways, policies and targets including ZEV mandate, heat pump installation targets, offshore wind ambition. Subject to ongoing JR scrutiny.
-[SUPERSEDED] The Carbon Budget Delivery Plan 2023 was superseded by the Carbon Budget and Growth Delivery Plan (CBGDP), published October 2025, which is now the Government plan for meeting the Fourth, Fifth and Sixth Carbon Budgets and the basis against which the CCC measures progress. The Net Zero Strategy 2021 element of this record is not itself superseded. A separate record for the CBGDP is queued.</t>
+[SUPERSEDED] The Carbon Budget Delivery Plan 2023 was superseded by the Carbon Budget and Growth Delivery Plan (CBGDP), published October 2025, which is now the Government plan for meeting the Fourth, Fifth and Sixth Carbon Budgets and the basis against which the CCC measures progress. The Net Zero Strategy 2021 element of this record is not itself superseded. The CBGDP is held as [POL-112].</t>
         </is>
       </c>
       <c r="O5" s="5" t="inlineStr">
@@ -10244,7 +10248,7 @@
       </c>
       <c r="P5" s="5" t="inlineStr">
         <is>
-          <t>September 2026</t>
+          <t>October 2026</t>
         </is>
       </c>
       <c r="Q5" s="6" t="inlineStr">
@@ -11273,7 +11277,11 @@
           <t>[LEG-001]; [LEG-002]</t>
         </is>
       </c>
-      <c r="J18" s="2" t="n"/>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>[POL-113] CCRA4-IA (May 2026)</t>
+        </is>
+      </c>
       <c r="K18" s="2" t="n"/>
       <c r="L18" s="2" t="n"/>
       <c r="M18" s="2" t="inlineStr">
@@ -11285,7 +11293,7 @@
         <is>
           <t>Third statutory CCRA covering 61 UK climate risks/opportunities across 5 themes. Forms basis for NAP3. CCRA4 will commence 2026–27 ahead of NAP4. Produced by CCC with government support.
 [VERSION HISTORY] CCRA3 (2022) is the third statutory assessment under CCA 2008 s.56. Previous versions: CCRA1 (2012), CCRA2 (2017). Covers 61 UK climate risks/opportunities across 5 themes. Forms basis for NAP3. CCRA4 will commence 2026–27 ahead of NAP4. Produced by CCC with government support. CCRA3 found adaptation progress 'insufficient' across most risk areas.
-[CURRENCY] The Fourth Independent Assessment of UK Climate Risk (CCRA4-IA) was published by the CCC on 20 May 2026 as "A Well-Adapted UK", with a Technical Report led by the Met Office. CCRA3 remains the current statutory assessment until CCRA4 is laid; the CCC has already moved its adaptation monitoring onto CCRA4-IA. A separate record for CCRA4-IA is queued.</t>
+[CURRENCY] The Fourth Independent Assessment of UK Climate Risk (CCRA4-IA) was published by the CCC on 20 May 2026 as "A Well-Adapted UK", with a Technical Report led by the Met Office. CCRA3 remains the current statutory assessment until CCRA4 is laid; the CCC has already moved its adaptation monitoring onto CCRA4-IA. CCRA4-IA is held as [POL-113]; the government must lay CCRA4 before Parliament by January 2027.</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
@@ -11295,7 +11303,7 @@
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>September 2026</t>
+          <t>October 2026</t>
         </is>
       </c>
       <c r="Q18" s="4" t="inlineStr">
@@ -13331,7 +13339,7 @@
       </c>
       <c r="N44" s="2" t="inlineStr">
         <is>
-          <t>Environment Agency statutory strategy setting long-term ambitions for a nation resilient to flooding and coastal change to 2100, with an accompanying action plan. Increasingly emphasises nature-based and catchment-scale solutions and adaptation; aligns with NAP3 [POL-002] and CCRA3 [POL-017]. [Themes: nature-based solutions; natural capital; ecosystem services]</t>
+          <t>Environment Agency statutory strategy setting long-term ambitions for a nation resilient to flooding and coastal change to 2100, with an accompanying action plan. Increasingly emphasises nature-based and catchment-scale solutions and adaptation; aligns with NAP3 [POL-002] and CCRA3 [POL-017]. [Themes: nature-based solutions; natural capital; ecosystem services] Regional example: Humber 2100+, a partnership of the Environment Agency and local authorities developing a long-term approach to tidal flood risk in the Humber estuary, where more than 500,000 people live in flood-prone areas and sea-level rise drives the need for an estuary-wide strategy ('Understanding tidal risk', July 2026). Held here rather than as a separate record (decision, 11 Sep 2026); compare [POL-100] TE2100.</t>
         </is>
       </c>
       <c r="O44" s="2" t="inlineStr">
@@ -13341,7 +13349,7 @@
       </c>
       <c r="P44" s="2" t="inlineStr">
         <is>
-          <t>June 2026</t>
+          <t>October 2026</t>
         </is>
       </c>
       <c r="Q44" s="4" t="inlineStr">
@@ -13724,7 +13732,7 @@
       </c>
       <c r="N49" s="5" t="inlineStr">
         <is>
-          <t>Sets out the government's planning policies for England and how they are applied in plan-making and decision-taking. The operative instrument mediating development against climate, nature and land-use objectives: mandatory housing targets (1.5m homes), 'grey belt' release, brownfield-first, reversal of the onshore-wind ban, biodiversity net gain, flood-risk and renewable-energy policy. Sits above local plans and complements the Land Use Framework [POL-009]. Further reform package consulted Dec 2025. [Themes: spatial planning; land-use change; development control]</t>
+          <t>Sets out the government's planning policies for England and how they are applied in plan-making and decision-taking. The operative instrument mediating development against climate, nature and land-use objectives: mandatory housing targets (1.5m homes), 'grey belt' release, brownfield-first, reversal of the onshore-wind ban, biodiversity net gain, flood-risk and renewable-energy policy. Sits above local plans and complements the Land Use Framework [POL-009]. Further reform package consulted Dec 2025. [Themes: spatial planning; land-use change; development control] Scope note: National Policy Statements made under the Planning Act 2008 [LEG-054] (e.g. ports, nuclear energy infrastructure) are not catalogued, as a class (decision, 10 Sep 2026); policy scans should not re-raise them.</t>
         </is>
       </c>
       <c r="O49" s="5" t="inlineStr">
@@ -13734,7 +13742,7 @@
       </c>
       <c r="P49" s="5" t="inlineStr">
         <is>
-          <t>June 2026</t>
+          <t>October 2026</t>
         </is>
       </c>
       <c r="Q49" s="6" t="inlineStr">
@@ -18651,6 +18659,423 @@
           <t>[INT-L-022] Aarhus Convention — UN/ECE Convention on Access to Information, Public Participation and Access to Justice in Environmental Matters</t>
         </is>
       </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="5" t="inlineStr">
+        <is>
+          <t>POL-112</t>
+        </is>
+      </c>
+      <c r="B111" s="5" t="inlineStr">
+        <is>
+          <t>Carbon Budget and Growth Delivery Plan (CBGDP)</t>
+        </is>
+      </c>
+      <c r="C111" s="5" t="inlineStr">
+        <is>
+          <t>CBGDP</t>
+        </is>
+      </c>
+      <c r="D111" s="5" t="inlineStr">
+        <is>
+          <t>Policy_Activity</t>
+        </is>
+      </c>
+      <c r="E111" s="12" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+      <c r="F111" s="5" t="inlineStr">
+        <is>
+          <t>Climate | Energy | Transport | Urban &amp; Buildings | Land Use &amp; Agriculture</t>
+        </is>
+      </c>
+      <c r="G111" s="5" t="inlineStr">
+        <is>
+          <t>2025 (published 29 Oct 2025, HC 1366; factsheets added Jun 2026)</t>
+        </is>
+      </c>
+      <c r="H111" s="5" t="inlineStr">
+        <is>
+          <t>Statutory</t>
+        </is>
+      </c>
+      <c r="I111" s="5" t="inlineStr">
+        <is>
+          <t>[LEG-001]; [LEG-003]</t>
+        </is>
+      </c>
+      <c r="J111" s="5" t="inlineStr">
+        <is>
+          <t>[POL-004] Carbon Budget Delivery Plan 2023 (superseded); [POL-018] Seventh Carbon Budget; [POL-114] CCC progress reports</t>
+        </is>
+      </c>
+      <c r="K111" s="5" t="n"/>
+      <c r="L111" s="5" t="n"/>
+      <c r="M111" s="5" t="inlineStr">
+        <is>
+          <t>[ORG-002] DESNZ</t>
+        </is>
+      </c>
+      <c r="N111" s="5" t="inlineStr">
+        <is>
+          <t>The government's report under section 14 of the Climate Change Act 2008 setting out how it will meet its statutory carbon budgets and secure the economic benefits of the transition; replaces the Carbon Budget Delivery Plan 2023 [POL-004] as the plan against which the CCC assesses progress. Main report with a technical annex and sector investor factsheets. The CCC indicator benchmarks in [IFW-02] were re-derived against it (indicators v18–v20).</t>
+        </is>
+      </c>
+      <c r="O111" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="P111" s="5" t="inlineStr">
+        <is>
+          <t>October 2026</t>
+        </is>
+      </c>
+      <c r="Q111" s="6" t="inlineStr">
+        <is>
+          <t>https://www.gov.uk/government/publications/carbon-budget-and-growth-delivery-plan-2025</t>
+        </is>
+      </c>
+      <c r="R111" s="6" t="inlineStr">
+        <is>
+          <t>[IFW-02]</t>
+        </is>
+      </c>
+      <c r="S111" s="6" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>POL-113</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>A Well-Adapted UK — Fourth Independent Assessment of UK Climate Risk (CCRA4-IA)</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>CCRA4-IA</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>Policy_Activity</t>
+        </is>
+      </c>
+      <c r="E112" s="11" t="inlineStr">
+        <is>
+          <t>Assessment / Evidence</t>
+        </is>
+      </c>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>Climate | Health | Nature &amp; Biodiversity | Water | Governance, Society &amp; Data</t>
+        </is>
+      </c>
+      <c r="G112" s="2" t="inlineStr">
+        <is>
+          <t>2026 (published 20 May 2026)</t>
+        </is>
+      </c>
+      <c r="H112" s="2" t="inlineStr">
+        <is>
+          <t>Statutory</t>
+        </is>
+      </c>
+      <c r="I112" s="2" t="inlineStr">
+        <is>
+          <t>[LEG-001]</t>
+        </is>
+      </c>
+      <c r="J112" s="2" t="inlineStr">
+        <is>
+          <t>[POL-017] CCRA3 2022; [POL-002] NAP3</t>
+        </is>
+      </c>
+      <c r="K112" s="2" t="n"/>
+      <c r="L112" s="2" t="n"/>
+      <c r="M112" s="2" t="inlineStr">
+        <is>
+          <t>[ORG-003] CCC</t>
+        </is>
+      </c>
+      <c r="N112" s="2" t="inlineStr">
+        <is>
+          <t>The CCC's statutory independent assessment of UK climate risk under section 57 of the Climate Change Act 2008, covering all four nations across 14 systems, assessed for 2°C of global warming by 2050 with 4°C by 2100 considered; prioritises eight highest-risk areas and, for the first time, proposes adaptation solutions. The Technical Report was led by the Met Office [ORG-017] (Prof Jason Lowe, Dr Mark Harrison, Rachel Perks) — a direct Met Office → policy channel. The UK Government must lay CCRA4 before Parliament by January 2027, followed by national adaptation programmes around 2028.</t>
+        </is>
+      </c>
+      <c r="O112" s="2" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="P112" s="2" t="inlineStr">
+        <is>
+          <t>October 2026</t>
+        </is>
+      </c>
+      <c r="Q112" s="4" t="inlineStr">
+        <is>
+          <t>https://www.theccc.org.uk/publication/a-well-adapted-uk/</t>
+        </is>
+      </c>
+      <c r="R112" s="4" t="inlineStr">
+        <is>
+          <t>[IFW-10]</t>
+        </is>
+      </c>
+      <c r="S112" s="4" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="5" t="inlineStr">
+        <is>
+          <t>POL-114</t>
+        </is>
+      </c>
+      <c r="B113" s="5" t="inlineStr">
+        <is>
+          <t>CCC progress reports to Parliament (annual emissions progress reports)</t>
+        </is>
+      </c>
+      <c r="C113" s="5" t="inlineStr">
+        <is>
+          <t>CCC Progress Reports</t>
+        </is>
+      </c>
+      <c r="D113" s="5" t="inlineStr">
+        <is>
+          <t>Policy_Activity</t>
+        </is>
+      </c>
+      <c r="E113" s="12" t="inlineStr">
+        <is>
+          <t>Assessment / Evidence</t>
+        </is>
+      </c>
+      <c r="F113" s="5" t="inlineStr">
+        <is>
+          <t>Climate | Energy | Transport | Land Use &amp; Agriculture | Governance, Society &amp; Data</t>
+        </is>
+      </c>
+      <c r="G113" s="5" t="inlineStr">
+        <is>
+          <t>Annual (latest: Progress in reducing emissions 2026, 24 Jun 2026)</t>
+        </is>
+      </c>
+      <c r="H113" s="5" t="inlineStr">
+        <is>
+          <t>Statutory</t>
+        </is>
+      </c>
+      <c r="I113" s="5" t="inlineStr">
+        <is>
+          <t>[LEG-001]</t>
+        </is>
+      </c>
+      <c r="J113" s="5" t="inlineStr">
+        <is>
+          <t>[POL-112] CBGDP; [POL-018] Seventh Carbon Budget</t>
+        </is>
+      </c>
+      <c r="K113" s="5" t="n"/>
+      <c r="L113" s="5" t="n"/>
+      <c r="M113" s="5" t="inlineStr">
+        <is>
+          <t>[ORG-003] CCC</t>
+        </is>
+      </c>
+      <c r="N113" s="5" t="inlineStr">
+        <is>
+          <t>The CCC's annual statutory report to Parliament on progress towards the carbon budgets and net zero, laid under section 36(1) of the Climate Change Act 2008: emissions trends, sectoral performance, and the credibility of government policy — the 2026 report assesses the CBGDP [POL-112]. Held as one record for the series, not one per year. The CCC's separate adaptation progress reporting is not covered here.</t>
+        </is>
+      </c>
+      <c r="O113" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="P113" s="5" t="inlineStr">
+        <is>
+          <t>October 2026</t>
+        </is>
+      </c>
+      <c r="Q113" s="6" t="inlineStr">
+        <is>
+          <t>https://www.theccc.org.uk/publication/progress-in-reducing-emissions-2026-report-to-parliament/</t>
+        </is>
+      </c>
+      <c r="R113" s="6" t="inlineStr">
+        <is>
+          <t>[IFW-02]</t>
+        </is>
+      </c>
+      <c r="S113" s="6" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>POL-115</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>Third Northern Ireland Climate Change Adaptation Programme (NICCAP3)</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>NICCAP3</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t>Policy_Activity</t>
+        </is>
+      </c>
+      <c r="E114" s="11" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+      <c r="F114" s="2" t="inlineStr">
+        <is>
+          <t>Climate | Water | Health | Nature &amp; Biodiversity | Governance, Society &amp; Data</t>
+        </is>
+      </c>
+      <c r="G114" s="2" t="inlineStr">
+        <is>
+          <t>2026 (published 19 Mar 2026; runs to 2029)</t>
+        </is>
+      </c>
+      <c r="H114" s="2" t="inlineStr">
+        <is>
+          <t>Statutory</t>
+        </is>
+      </c>
+      <c r="I114" s="2" t="inlineStr">
+        <is>
+          <t>[LEG-001]</t>
+        </is>
+      </c>
+      <c r="J114" s="2" t="inlineStr">
+        <is>
+          <t>[POL-002] NAP3 (England); [POL-017] CCRA3 2022</t>
+        </is>
+      </c>
+      <c r="K114" s="2" t="n"/>
+      <c r="L114" s="2" t="n"/>
+      <c r="M114" s="2" t="inlineStr">
+        <is>
+          <t>[ORG-036] Northern Ireland Executive (DAERA)</t>
+        </is>
+      </c>
+      <c r="N114" s="2" t="inlineStr">
+        <is>
+          <t>Northern Ireland's statutory adaptation programme under section 60 of the Climate Change Act 2008, responding to the risks identified in CCRA3: over 280 actions from across NI Executive departments and wider stakeholders, covering flooding, heatwaves, severe storms and other climate impacts. Northern Ireland counterpart of NAP3 [POL-002].</t>
+        </is>
+      </c>
+      <c r="O114" s="2" t="inlineStr">
+        <is>
+          <t>Northern Ireland</t>
+        </is>
+      </c>
+      <c r="P114" s="2" t="inlineStr">
+        <is>
+          <t>October 2026</t>
+        </is>
+      </c>
+      <c r="Q114" s="4" t="inlineStr">
+        <is>
+          <t>https://www.daera-ni.gov.uk/publications/third-northern-ireland-climate-change-adaptation-programme</t>
+        </is>
+      </c>
+      <c r="R114" s="4" t="n"/>
+      <c r="S114" s="4" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="5" t="inlineStr">
+        <is>
+          <t>POL-116</t>
+        </is>
+      </c>
+      <c r="B115" s="5" t="inlineStr">
+        <is>
+          <t>Scotland's Climate Change Plan 2026–2040</t>
+        </is>
+      </c>
+      <c r="C115" s="5" t="inlineStr">
+        <is>
+          <t>CCP 2026–40</t>
+        </is>
+      </c>
+      <c r="D115" s="5" t="inlineStr">
+        <is>
+          <t>Policy_Activity</t>
+        </is>
+      </c>
+      <c r="E115" s="12" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+      <c r="F115" s="5" t="inlineStr">
+        <is>
+          <t>Climate | Energy | Transport | Land Use &amp; Agriculture | Urban &amp; Buildings</t>
+        </is>
+      </c>
+      <c r="G115" s="5" t="inlineStr">
+        <is>
+          <t>2026 (final plan published 24 Mar 2026; draft 6 Nov 2025)</t>
+        </is>
+      </c>
+      <c r="H115" s="5" t="inlineStr">
+        <is>
+          <t>Statutory</t>
+        </is>
+      </c>
+      <c r="I115" s="5" t="inlineStr">
+        <is>
+          <t>[LEG-058]</t>
+        </is>
+      </c>
+      <c r="J115" s="5" t="inlineStr">
+        <is>
+          <t>[POL-112] CBGDP (UK)</t>
+        </is>
+      </c>
+      <c r="K115" s="5" t="n"/>
+      <c r="L115" s="5" t="n"/>
+      <c r="M115" s="5" t="inlineStr">
+        <is>
+          <t>[ORG-034] Scottish Government</t>
+        </is>
+      </c>
+      <c r="N115" s="5" t="inlineStr">
+        <is>
+          <t>Scotland's statutory plan setting out policies and proposals to meet its first three carbon budgets (2026–2030, 2031–2035, 2036–2040) on the path to net zero by 2045, with sectoral contributions, costs and benefits, and just-transition measures. The CCC assessed the draft (Feb 2026) as credible or low-risk for 91% of the reductions needed in the first budget, with significant risks for later budgets. Scottish counterpart of the UK CBGDP [POL-112].</t>
+        </is>
+      </c>
+      <c r="O115" s="5" t="inlineStr">
+        <is>
+          <t>Scotland</t>
+        </is>
+      </c>
+      <c r="P115" s="5" t="inlineStr">
+        <is>
+          <t>October 2026</t>
+        </is>
+      </c>
+      <c r="Q115" s="6" t="inlineStr">
+        <is>
+          <t>https://www.gov.scot/publications/scotlands-climate-change-plan-2026-2040-annexes/</t>
+        </is>
+      </c>
+      <c r="R115" s="6" t="n"/>
+      <c r="S115" s="6" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:N1"/>
@@ -19728,7 +20153,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H229"/>
+  <dimension ref="A1:H233"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="32" min="1" max="1"/>
@@ -29041,14 +29466,214 @@
       </c>
     </row>
     <row r="229" ht="27.75" customHeight="1" s="32">
-      <c r="A229" s="2" t="n"/>
-      <c r="B229" s="2" t="n"/>
-      <c r="C229" s="2" t="n"/>
-      <c r="D229" s="2" t="n"/>
-      <c r="E229" s="2" t="n"/>
-      <c r="F229" s="2" t="n"/>
-      <c r="G229" s="2" t="n"/>
-      <c r="H229" s="2" t="n"/>
+      <c r="A229" s="2" t="inlineStr">
+        <is>
+          <t>POL-112</t>
+        </is>
+      </c>
+      <c r="B229" s="2" t="inlineStr">
+        <is>
+          <t>Carbon Budget and Growth Delivery Plan (CBGDP)</t>
+        </is>
+      </c>
+      <c r="C229" s="2" t="inlineStr">
+        <is>
+          <t>CBGDP</t>
+        </is>
+      </c>
+      <c r="D229" s="2" t="inlineStr">
+        <is>
+          <t>Policy_Activity</t>
+        </is>
+      </c>
+      <c r="E229" s="2" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+      <c r="F229" s="2" t="inlineStr">
+        <is>
+          <t>Climate | Energy | Transport | Urban &amp; Buildings | Land Use &amp; Agriculture</t>
+        </is>
+      </c>
+      <c r="G229" s="2" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="H229" s="2" t="inlineStr">
+        <is>
+          <t>Policies &amp; Activities</t>
+        </is>
+      </c>
+    </row>
+    <row r="230" ht="27.75" customHeight="1" s="32">
+      <c r="A230" s="2" t="inlineStr">
+        <is>
+          <t>POL-113</t>
+        </is>
+      </c>
+      <c r="B230" s="2" t="inlineStr">
+        <is>
+          <t>A Well-Adapted UK — Fourth Independent Assessment of UK Climate Risk (CCRA4-IA)</t>
+        </is>
+      </c>
+      <c r="C230" s="2" t="inlineStr">
+        <is>
+          <t>CCRA4-IA</t>
+        </is>
+      </c>
+      <c r="D230" s="2" t="inlineStr">
+        <is>
+          <t>Policy_Activity</t>
+        </is>
+      </c>
+      <c r="E230" s="2" t="inlineStr">
+        <is>
+          <t>Assessment / Evidence</t>
+        </is>
+      </c>
+      <c r="F230" s="2" t="inlineStr">
+        <is>
+          <t>Climate | Health | Nature &amp; Biodiversity | Water | Governance, Society &amp; Data</t>
+        </is>
+      </c>
+      <c r="G230" s="2" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="H230" s="2" t="inlineStr">
+        <is>
+          <t>Policies &amp; Activities</t>
+        </is>
+      </c>
+    </row>
+    <row r="231" ht="27.75" customHeight="1" s="32">
+      <c r="A231" s="2" t="inlineStr">
+        <is>
+          <t>POL-114</t>
+        </is>
+      </c>
+      <c r="B231" s="2" t="inlineStr">
+        <is>
+          <t>CCC progress reports to Parliament (annual emissions progress reports)</t>
+        </is>
+      </c>
+      <c r="C231" s="2" t="inlineStr">
+        <is>
+          <t>CCC Progress Reports</t>
+        </is>
+      </c>
+      <c r="D231" s="2" t="inlineStr">
+        <is>
+          <t>Policy_Activity</t>
+        </is>
+      </c>
+      <c r="E231" s="2" t="inlineStr">
+        <is>
+          <t>Assessment / Evidence</t>
+        </is>
+      </c>
+      <c r="F231" s="2" t="inlineStr">
+        <is>
+          <t>Climate | Energy | Transport | Land Use &amp; Agriculture | Governance, Society &amp; Data</t>
+        </is>
+      </c>
+      <c r="G231" s="2" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="H231" s="2" t="inlineStr">
+        <is>
+          <t>Policies &amp; Activities</t>
+        </is>
+      </c>
+    </row>
+    <row r="232" ht="27.75" customHeight="1" s="32">
+      <c r="A232" s="2" t="inlineStr">
+        <is>
+          <t>POL-115</t>
+        </is>
+      </c>
+      <c r="B232" s="2" t="inlineStr">
+        <is>
+          <t>Third Northern Ireland Climate Change Adaptation Programme (NICCAP3)</t>
+        </is>
+      </c>
+      <c r="C232" s="2" t="inlineStr">
+        <is>
+          <t>NICCAP3</t>
+        </is>
+      </c>
+      <c r="D232" s="2" t="inlineStr">
+        <is>
+          <t>Policy_Activity</t>
+        </is>
+      </c>
+      <c r="E232" s="2" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+      <c r="F232" s="2" t="inlineStr">
+        <is>
+          <t>Climate | Water | Health | Nature &amp; Biodiversity | Governance, Society &amp; Data</t>
+        </is>
+      </c>
+      <c r="G232" s="2" t="inlineStr">
+        <is>
+          <t>Northern Ireland</t>
+        </is>
+      </c>
+      <c r="H232" s="2" t="inlineStr">
+        <is>
+          <t>Policies &amp; Activities</t>
+        </is>
+      </c>
+    </row>
+    <row r="233" ht="27.75" customHeight="1" s="32">
+      <c r="A233" s="2" t="inlineStr">
+        <is>
+          <t>POL-116</t>
+        </is>
+      </c>
+      <c r="B233" s="2" t="inlineStr">
+        <is>
+          <t>Scotland's Climate Change Plan 2026–2040</t>
+        </is>
+      </c>
+      <c r="C233" s="2" t="inlineStr">
+        <is>
+          <t>CCP 2026–40</t>
+        </is>
+      </c>
+      <c r="D233" s="2" t="inlineStr">
+        <is>
+          <t>Policy_Activity</t>
+        </is>
+      </c>
+      <c r="E233" s="2" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+      <c r="F233" s="2" t="inlineStr">
+        <is>
+          <t>Climate | Energy | Transport | Land Use &amp; Agriculture | Urban &amp; Buildings</t>
+        </is>
+      </c>
+      <c r="G233" s="2" t="inlineStr">
+        <is>
+          <t>Scotland</t>
+        </is>
+      </c>
+      <c r="H233" s="2" t="inlineStr">
+        <is>
+          <t>Policies &amp; Activities</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
@@ -29063,7 +29688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="32" min="1" max="1"/>
@@ -29091,7 +29716,7 @@
         </is>
       </c>
       <c r="B2" s="17" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="32">
@@ -29418,6 +30043,72 @@
         </is>
       </c>
       <c r="D21" t="inlineStr">
+        <is>
+          <t>Cowork (Claude)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>v30</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>v30: Decided edits from the September queue triage (handover Open work 2), approved by Jonathan 6 Oct 2026. LEG-025 Water Resources Act 1991: drought orders and drought permits (Part II Ch. III, ss.73–81, s.79A) described, with the decision not to catalogue individual orders. LEG-023 Water Act 2014: ss.27–28 (WRMP resilience; frequency of WRMPs and drought plans) noted, pointing to LEG-025 for orders and permits. ORG-004 JNCC: the 'Nature, Evidence and Action' Signpost report series added as a mention and link (decision 11 Sep 2026: mention, not records). POL-050 NPPF: scope note that National Policy Statements are excluded as a class (decision 10 Sep 2026). LEG-013 Status: Royal Assent date verified as 24 Feb 2025 (was 'Jan 2025'). All verified at legislation.gov.uk and jncc.gov.uk on 6 Oct 2026. Humber 2100+ / POL-045 not done: still awaiting a decision.</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Cowork (Claude)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>v31</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>v31: POL-045 FCERM Strategy gains a sentence on Humber 2100+ (Environment Agency with local authorities; 'Humber 2100+ Understanding tidal risk', gov.uk, 7 Jul 2026, updated 20 Jul 2026), folded in rather than held as a record, per the 11 Sep 2026 decision; approved by Jonathan 6 Oct 2026.</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Cowork (Claude)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>v32</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>v32: The five 'pending' rows from the 17 Sep 2026 framework-currency check, approved by Jonathan 6 Oct 2026. NEW: POL-112 Carbon Budget and Growth Delivery Plan (DESNZ, 29 Oct 2025, CCA 2008 s.14 report); POL-113 A Well-Adapted UK — CCRA4-IA (CCC, 20 May 2026, s.57; Met Office-led Technical Report); POL-114 CCC progress reports to Parliament (annual, s.36(1)) — one record for the series, not per year, by decision; POL-115 NICCAP3 (DAERA, 19 Mar 2026, s.60); POL-116 Scotland's Climate Change Plan 2026–2040 (final 24 Mar 2026; statutory basis Climate Change (Scotland) Act 2009 s.35 inherited, not re-read). EDITS: POL-004 points to POL-112 (resolves the 'CBGDP may supersede POL-004' investigate row); POL-017 points to POL-113 and stays the current statutory CCRA until CCRA4 is laid (due by Jan 2027). Verified at gov.uk, theccc.org.uk, daera-ni.gov.uk and gov.scot on 6 Oct 2026.</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
         <is>
           <t>Cowork (Claude)</t>
         </is>

</xml_diff>

<commit_message>
Indicators v28 / UK v33: MCCIP indicator block (IFW-12, IND-M-001–016)
- New 'MCCIP Indicators' sheet and register row IFW-12: the 16 physical-environment and
  ecosystem-change topics of the MCCIP Impacts Hub, read at source 6 Oct 2026.
- Climate scores checked against outputs_other/CLIMATE_SCORE_METHOD.md (1/2/3 = 3/3/10),
  with rule G siblings cited in each rationale.
- POL-049 links to IFW-12; finder gains the MCCIP framework and filter.
- Counts updated to 1,001 records across docs; queue and Open work resolved.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AXpUr5Jv7F4hv6YdhfHEwx
</commit_message>
<xml_diff>
--- a/Data/canonical_files/uk_climate_nature_governance.xlsx
+++ b/Data/canonical_files/uk_climate_nature_governance.xlsx
@@ -13657,7 +13657,7 @@
       </c>
       <c r="P48" s="2" t="inlineStr">
         <is>
-          <t>June 2026</t>
+          <t>October 2026</t>
         </is>
       </c>
       <c r="Q48" s="4" t="inlineStr">
@@ -13665,7 +13665,11 @@
           <t>https://www.mccip.org.uk/</t>
         </is>
       </c>
-      <c r="R48" s="4" t="n"/>
+      <c r="R48" s="4" t="inlineStr">
+        <is>
+          <t>[IFW-12]</t>
+        </is>
+      </c>
       <c r="S48" s="4" t="inlineStr">
         <is>
           <t>[INT-O-027] Arctic Monitoring and Assessment Programme; [INT-P-032] IPCC Special Report on the Ocean and Cryosphere in a Changing Climate (SROCC) 2019; [INT-P-033] UN Decade of Ocean Science for Sustainable Development (2021-2030)</t>
@@ -29688,7 +29692,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="32" min="1" max="1"/>
@@ -29716,7 +29720,7 @@
         </is>
       </c>
       <c r="B2" s="17" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="32">
@@ -29731,6 +29735,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="42" customHeight="1" s="32">
       <c r="A5" s="31" t="inlineStr">
         <is>
@@ -30109,6 +30114,28 @@
         </is>
       </c>
       <c r="D24" t="inlineStr">
+        <is>
+          <t>Cowork (Claude)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>v33</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>v33: POL-049 MCCIP Indicator_Frameworks gains [IFW-12], the MCCIP indicator block added in indicators v28.</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
         <is>
           <t>Cowork (Claude)</t>
         </is>

</xml_diff>

<commit_message>
UK v34: correct LEG-003 Carbon Budget Order link
LEG-003 linked to uksi/2021/1059, which resolves to wsi/2021/1059 (a
revoked Welsh commencement order). Corrected to uksi/2021/750, The Carbon
Budget Order 2021, verified against legislation.gov.uk data.xml. Found by
check_legislation_links.py on its first live run for this record.

- Title cache: verified entries for LEG-003 and LEG-049
- Handover and README: UK v34; LEG-003/049 removed from Open work item 2
- Dashboards and exports rebuilt by finalise.py

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AXpUr5Jv7F4hv6YdhfHEwx
</commit_message>
<xml_diff>
--- a/Data/canonical_files/uk_climate_nature_governance.xlsx
+++ b/Data/canonical_files/uk_climate_nature_governance.xlsx
@@ -4729,7 +4729,7 @@
       </c>
       <c r="N4" s="4" t="inlineStr">
         <is>
-          <t>https://www.legislation.gov.uk/uksi/2021/1059/contents</t>
+          <t>https://www.legislation.gov.uk/uksi/2021/750/contents</t>
         </is>
       </c>
       <c r="O4" s="2" t="n"/>
@@ -29692,7 +29692,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="32" min="1" max="1"/>
@@ -29719,8 +29719,10 @@
           <t>Version</t>
         </is>
       </c>
-      <c r="B2" s="17" t="n">
-        <v>33</v>
+      <c r="B2" s="17" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="32">
@@ -29731,11 +29733,10 @@
       </c>
       <c r="B3" s="17" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-    </row>
-    <row r="4"/>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
     <row r="5" ht="42" customHeight="1" s="32">
       <c r="A5" s="31" t="inlineStr">
         <is>
@@ -30136,6 +30137,28 @@
         </is>
       </c>
       <c r="D25" t="inlineStr">
+        <is>
+          <t>Cowork (Claude)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>v34</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>v34: [LEG-003] Carbon Budget Orders — Link corrected from uksi/2021/1059 (resolves to wsi/2021/1059, the Historic Environment (Wales) Act 2016 (Commencement No. 2) Order 2021, revoked) to uksi/2021/750, The Carbon Budget Order 2021; verified against legislation.gov.uk data.xml 7 Oct 2026. Found by check_legislation_links.py on its first live run for this record.</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
         <is>
           <t>Cowork (Claude)</t>
         </is>

</xml_diff>